<commit_message>
Fill real chapa-fechada and fita prices, regenerate real partial budget
User provided and confirmed real per-sheet (not per-m2) and per-meter
edge-tape prices for the 7 already-known references. Regenerated
orcamento_final.xlsx against the real Quarto Maria extraction: 2 of
those 7 references actually appear in this project (the other 5 exist
in the price table but aren't used here), giving a partial material
cost of R$1.998,93 -> R$5.517,33 after markup. Verified by hand:
matches the script's own printed total exactly. 43 items (14 more
chapa/fita references plus all hardware) remain unpriced and correctly
excluded from the total.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XB6sVbz8mNsHFq3uDSYMc1
</commit_message>
<xml_diff>
--- a/orcamento-marcenaria/output/orcamento_final.xlsx
+++ b/orcamento-marcenaria/output/orcamento_final.xlsx
@@ -16,10 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="$#,##0.00;($#,##0.00);&quot;-&quot;"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="$#,##0.00;($#,##0.00);&quot;-&quot;"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -115,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,10 +127,13 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -588,432 +592,481 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>1.0394.18.Berneck.Unicolors Metallic Suede TX.MDF</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>4.508</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>539.9</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>539.9</v>
+      </c>
+    </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>2.2018.18.Duratex.Essencial.Rosa Infinito.MDF</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>0.1725</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>519.9</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>519.9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Fita de Borda</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Referencia</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Metros Total</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Preco/Metro (R$)</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>Custo (R$)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>1.0394.18.Berneck.Unicolors Metallic Suede TX.MDF</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>21.68</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>778.312</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>2.2018.18.Duratex.Essencial.Rosa Infinito.MDF</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>4.888</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>160.8152</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Ferragens / Componentes</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Descricao</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Referencia</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Custo (R$)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>Custo Material Total</t>
         </is>
       </c>
-      <c r="B18" s="9" t="n">
+      <c r="B22" s="12">
+        <f>SUM(F10:F11)+SUM(D15:D16)+SUM(C20:C19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>Preco Venda Material (x Markup)</t>
+        </is>
+      </c>
+      <c r="B23" s="12">
+        <f>B22*$B$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Mao de Obra</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="n">
         <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>Preco Venda Material (x Markup)</t>
-        </is>
-      </c>
-      <c r="B19" s="9">
-        <f>B18*$B$5</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>Mao de Obra</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>TOTAL GERAL</t>
-        </is>
-      </c>
-      <c r="B21" s="11">
-        <f>B19+B20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t>Pendencias sem preco na tabela (47) -- NAO incluidas no total:</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 2.2035.18.Duratex.Essencial.Rosa Infinito.MDF ((chapa))</t>
-        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
+          <t>TOTAL GERAL</t>
+        </is>
+      </c>
+      <c r="B25" s="14">
+        <f>B23+B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t>Pendencias sem preco na tabela (43) -- NAO incluidas no total:</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 2.2035.18.Duratex.Essencial.Rosa Infinito.MDF ((chapa))</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
+        <is>
           <t xml:space="preserve">  SEM_PRECO_FITA_NA_TABELA: 2.2035.18.Duratex.Essencial.Rosa Infinito.MDF ((fita de borda))</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 2.2008.18.Branco.MDF ((chapa))</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_FITA_NA_TABELA: 2.2008.18.Branco.MDF ((fita de borda))</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 2.2015.9.Branco.MDF ((chapa))</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_FITA_NA_TABELA: 2.2015.9.Branco.MDF ((fita de borda))</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="13" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 2.2033.18.Branco.MDF ((chapa))</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="13" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_FITA_NA_TABELA: 2.2033.18.Branco.MDF ((fita de borda))</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 1.0394.18.Berneck.Unicolors Metallic Suede TX.MDF ((chapa))</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SEM_PRECO_FITA_NA_TABELA: 1.0394.18.Berneck.Unicolors Metallic Suede TX.MDF ((fita de borda))</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 2.0160.18.Branco.MDF ((chapa))</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_FITA_NA_TABELA: 2.0160.18.Branco.MDF ((fita de borda))</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="13" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 2.2029.18.Branco.MDF ((chapa))</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_FITA_NA_TABELA: 2.2029.18.Branco.MDF ((fita de borda))</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 2.2008.18.Duratex.Essencial.Rosa Infinito.MDF ((chapa))</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_FITA_NA_TABELA: 2.2008.18.Duratex.Essencial.Rosa Infinito.MDF ((fita de borda))</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="13" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 1.0854.18.Duratex.Essencial.Rosa Infinito.MDF ((chapa))</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="13" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_FITA_NA_TABELA: 1.0854.18.Duratex.Essencial.Rosa Infinito.MDF ((fita de borda))</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 2.2018.18.Duratex.Essencial.Rosa Infinito.MDF ((chapa))</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SEM_PRECO_FITA_NA_TABELA: 2.2018.18.Duratex.Essencial.Rosa Infinito.MDF ((fita de borda))</t>
-        </is>
-      </c>
-    </row>
     <row r="44">
-      <c r="A44" s="13" t="inlineStr">
+      <c r="A44" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 2.2015.18.Duratex.Essencial.Rosa Infinito.MDF ((chapa))</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="13" t="inlineStr">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_FITA_NA_TABELA: 2.2015.18.Duratex.Essencial.Rosa Infinito.MDF ((fita de borda))</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="13" t="inlineStr">
+      <c r="A46" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 2.2033.18.Duratex.Essencial.Rosa Infinito.MDF ((chapa))</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="13" t="inlineStr">
+      <c r="A47" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_FITA_NA_TABELA: 2.2033.18.Duratex.Essencial.Rosa Infinito.MDF ((fita de borda))</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="13" t="inlineStr">
+      <c r="A48" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 1.0260.18.Branco.MDF ((chapa))</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="13" t="inlineStr">
+      <c r="A49" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_FITA_NA_TABELA: 1.0260.18.Branco.MDF ((fita de borda))</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="13" t="inlineStr">
+      <c r="A50" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_CHAPA_NA_TABELA: 2.0109.18.Duratex.Essencial.Rosa Infinito.MDF ((chapa))</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="13" t="inlineStr">
+      <c r="A51" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_FITA_NA_TABELA: 2.0109.18.Duratex.Essencial.Rosa Infinito.MDF ((fita de borda))</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="13" t="inlineStr">
+      <c r="A52" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.1029.000 (Suporte)</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="13" t="inlineStr">
+      <c r="A53" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.1029.000 (Suporte)</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="13" t="inlineStr">
+      <c r="A54" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.1029.000 (Suporte)</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="13" t="inlineStr">
+      <c r="A55" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.1029.000 (Suporte)</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="13" t="inlineStr">
+      <c r="A56" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 1.1089.450 (Corrediça Telescópica 450)</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="13" t="inlineStr">
+      <c r="A57" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 1.1089.500 (Corrediça Telescópica 500)</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="13" t="inlineStr">
+      <c r="A58" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 1.1086.000 (Dobradiça Aço s/ Amort. Reta / Baixa)</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="13" t="inlineStr">
+      <c r="A59" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.0095C.734.Branco (Gaveta Interna c/ Contra Frente)</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="13" t="inlineStr">
+      <c r="A60" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.0095C.734.Branco (Gaveta Interna c/ Contra Frente)</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="13" t="inlineStr">
+      <c r="A61" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.0095C.734.Branco (Gaveta Interna c/ Contra Frente)</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="13" t="inlineStr">
+      <c r="A62" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.0295.720.Branco (Sapateira com contra-frente)</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="13" t="inlineStr">
+      <c r="A63" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.0295.720.Branco (Sapateira com contra-frente)</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="13" t="inlineStr">
+      <c r="A64" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.0095C.734.Branco (Gaveta Interna c/ Contra Frente)</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="13" t="inlineStr">
+      <c r="A65" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.0095C.734.Branco (Gaveta Interna c/ Contra Frente)</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="13" t="inlineStr">
+      <c r="A66" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.0095C.734.Branco (Gaveta Interna c/ Contra Frente)</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="13" t="inlineStr">
+      <c r="A67" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.0295.720.Branco (Sapateira com contra-frente)</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="13" t="inlineStr">
+      <c r="A68" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.0295.720.Branco (Sapateira com contra-frente)</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="13" t="inlineStr">
+      <c r="A69" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: 2.0135.30.Duratex.Essencial.Rosa Infinito (Fechamento p/ Armário)</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="13" t="inlineStr">
+      <c r="A70" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEM_PRECO_NA_TABELA: Porta Provençal Configurável (Processo de Fabricação)</t>
         </is>

</xml_diff>

<commit_message>
Decouple Divisor de Markup from the % breakdown -- fixed but editable
Per user request, the markup divisor no longer recalculates when the
5 underlying percentages or any price changes -- it's its own blue
editable cell, initialized from the confirmed config value. The %
breakdown rows stay visible as reference/documentation but are
explicitly labeled as not feeding the divisor. Regenerated the real
Quarto Maria budget: total unchanged (R\$28.837,34), confirmed
Preco Venda Material's formula now references the fixed $B$11 cell
directly rather than a formula chain from the percentages.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XB6sVbz8mNsHFq3uDSYMc1
</commit_message>
<xml_diff>
--- a/orcamento-marcenaria/output/orcamento_final.xlsx
+++ b/orcamento-marcenaria/output/orcamento_final.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="167" formatCode="0.0"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +39,12 @@
     <font>
       <name val="Arial"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -121,25 +127,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -505,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -540,187 +546,173 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
+          <t>Composicao do markup (referencia -- nao alimenta o Divisor abaixo):</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
           <t>% Custo Fixo</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B6" s="5" t="n">
         <v>0.3377</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>% Impostos</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B7" s="5" t="n">
         <v>0.09</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>% Comissao Fabrica</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B8" s="5" t="n">
         <v>0.01</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>% Comissao Vendas (faixa aplicada)</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B9" s="5" t="n">
         <v>0.05</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>% Lucro</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B10" s="5" t="n">
         <v>0.15</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Divisor de Markup</t>
-        </is>
-      </c>
-      <c r="B10" s="5">
-        <f>1/(1-(B5+B6+B7+B8+B9))</f>
-        <v/>
-      </c>
-    </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Divisor de Markup (fixo, editavel)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>2.760143527463427</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>(nao muda automaticamente com os % acima ou com os precos -- edite direto aqui)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>% Perda de Corte</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B12" s="7" t="n">
         <v>0.15</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Area Util da Chapa (m2)</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B13" s="6" t="n">
         <v>5.032500000000001</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Custo Hora Mao de Obra (R$)</t>
         </is>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B14" s="8" t="n">
         <v>32.25</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Horas Estimadas</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B15" s="9" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Chapas de MDF</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>Acabamento</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Area Total (m2)</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>Area c/ Perda (m2)</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>Num Chapas</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Preco/Chapa (R$)</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr">
+      <c r="F18" s="11" t="inlineStr">
         <is>
           <t>Custo (R$)</t>
         </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>18mm Duratex.Essencial.Rosa Infinito</t>
-        </is>
-      </c>
-      <c r="B18" s="13" t="n">
-        <v>3.96</v>
-      </c>
-      <c r="C18" s="13">
-        <f>B18*(1+$B$11)</f>
-        <v/>
-      </c>
-      <c r="D18" s="12">
-        <f>ROUNDUP(C18/$B$12,0)</f>
-        <v/>
-      </c>
-      <c r="E18" s="14" t="n">
-        <v>591.9</v>
-      </c>
-      <c r="F18" s="15">
-        <f>D18*E18</f>
-        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>18mm Branco</t>
+          <t>18mm Duratex.Essencial.Rosa Infinito</t>
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>10.02</v>
+        <v>3.96</v>
       </c>
       <c r="C19" s="13">
-        <f>B19*(1+$B$11)</f>
+        <f>B19*(1+$B$12)</f>
         <v/>
       </c>
       <c r="D19" s="12">
-        <f>ROUNDUP(C19/$B$12,0)</f>
+        <f>ROUNDUP(C19/$B$13,0)</f>
         <v/>
       </c>
       <c r="E19" s="14" t="n">
-        <v>334.9</v>
+        <v>591.9</v>
       </c>
       <c r="F19" s="15">
         <f>D19*E19</f>
@@ -730,22 +722,22 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>9mm Branco</t>
+          <t>18mm Branco</t>
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>3.96</v>
+        <v>10.02</v>
       </c>
       <c r="C20" s="13">
-        <f>B20*(1+$B$11)</f>
+        <f>B20*(1+$B$12)</f>
         <v/>
       </c>
       <c r="D20" s="12">
-        <f>ROUNDUP(C20/$B$12,0)</f>
+        <f>ROUNDUP(C20/$B$13,0)</f>
         <v/>
       </c>
       <c r="E20" s="14" t="n">
-        <v>253.9</v>
+        <v>334.9</v>
       </c>
       <c r="F20" s="15">
         <f>D20*E20</f>
@@ -755,85 +747,93 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>18mm Berneck.Unicolors Metallic Suede TX</t>
+          <t>9mm Branco</t>
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>3.92</v>
+        <v>3.96</v>
       </c>
       <c r="C21" s="13">
-        <f>B21*(1+$B$11)</f>
+        <f>B21*(1+$B$12)</f>
         <v/>
       </c>
       <c r="D21" s="12">
-        <f>ROUNDUP(C21/$B$12,0)</f>
+        <f>ROUNDUP(C21/$B$13,0)</f>
         <v/>
       </c>
       <c r="E21" s="14" t="n">
-        <v>539.9</v>
+        <v>253.9</v>
       </c>
       <c r="F21" s="15">
         <f>D21*E21</f>
         <v/>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>18mm Berneck.Unicolors Metallic Suede TX</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="C22" s="13">
+        <f>B22*(1+$B$12)</f>
+        <v/>
+      </c>
+      <c r="D22" s="12">
+        <f>ROUNDUP(C22/$B$13,0)</f>
+        <v/>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>539.9</v>
+      </c>
+      <c r="F22" s="15">
+        <f>D22*E22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Fita de Borda</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>Acabamento</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Metros Total</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>Preco/Metro (R$)</t>
         </is>
       </c>
-      <c r="D24" s="11" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Custo (R$)</t>
         </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>18mm Duratex.Essencial.Rosa Infinito</t>
-        </is>
-      </c>
-      <c r="B25" s="13" t="n">
-        <v>49.6164</v>
-      </c>
-      <c r="C25" s="14" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="D25" s="15">
-        <f>B25*C25</f>
-        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>18mm Branco</t>
+          <t>18mm Duratex.Essencial.Rosa Infinito</t>
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>74.248</v>
+        <v>49.6164</v>
       </c>
       <c r="C26" s="14" t="n">
-        <v>26.9</v>
+        <v>32.9</v>
       </c>
       <c r="D26" s="15">
         <f>B26*C26</f>
@@ -843,14 +843,14 @@
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>9mm Branco</t>
+          <t>18mm Branco</t>
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>12.604</v>
+        <v>74.248</v>
       </c>
       <c r="C27" s="14" t="n">
-        <v>79.90000000000001</v>
+        <v>26.9</v>
       </c>
       <c r="D27" s="15">
         <f>B27*C27</f>
@@ -860,74 +860,69 @@
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>18mm Berneck.Unicolors Metallic Suede TX</t>
+          <t>9mm Branco</t>
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>21.68</v>
+        <v>12.604</v>
       </c>
       <c r="C28" s="14" t="n">
-        <v>35.9</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="D28" s="15">
         <f>B28*C28</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="10" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>18mm Berneck.Unicolors Metallic Suede TX</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="n">
+        <v>21.68</v>
+      </c>
+      <c r="C29" s="14" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="D29" s="15">
+        <f>B29*C29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>Ferragens / Componentes</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>Descricao</t>
         </is>
       </c>
-      <c r="B31" s="11" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>Referencia</t>
         </is>
       </c>
-      <c r="C31" s="11" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>Preco Unitario (R$)</t>
         </is>
       </c>
-      <c r="D31" s="11" t="inlineStr">
+      <c r="D32" s="11" t="inlineStr">
         <is>
           <t>Quantidade</t>
         </is>
       </c>
-      <c r="E31" s="11" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>Custo (R$)</t>
         </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="12" t="inlineStr">
-        <is>
-          <t>Suporte</t>
-        </is>
-      </c>
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t>2.1029.000</t>
-        </is>
-      </c>
-      <c r="C32" s="14" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="D32" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="E32" s="15">
-        <f>C32*D32</f>
-        <v/>
       </c>
     </row>
     <row r="33">
@@ -999,19 +994,19 @@
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
-          <t>Corrediça Telescópica 450</t>
+          <t>Suporte</t>
         </is>
       </c>
       <c r="B36" s="12" t="inlineStr">
         <is>
-          <t>1.1089.450</t>
+          <t>2.1029.000</t>
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>70</v>
+        <v>9.9</v>
       </c>
       <c r="D36" s="12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E36" s="15">
         <f>C36*D36</f>
@@ -1021,19 +1016,19 @@
     <row r="37">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>Corrediça Telescópica 500</t>
+          <t>Corrediça Telescópica 450</t>
         </is>
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>1.1089.500</t>
+          <t>1.1089.450</t>
         </is>
       </c>
       <c r="C37" s="14" t="n">
-        <v>76.5</v>
+        <v>70</v>
       </c>
       <c r="D37" s="12" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E37" s="15">
         <f>C37*D37</f>
@@ -1043,19 +1038,19 @@
     <row r="38">
       <c r="A38" s="12" t="inlineStr">
         <is>
-          <t>Dobradiça Aço s/ Amort. Reta / Baixa</t>
+          <t>Corrediça Telescópica 500</t>
         </is>
       </c>
       <c r="B38" s="12" t="inlineStr">
         <is>
-          <t>1.1086.000</t>
+          <t>1.1089.500</t>
         </is>
       </c>
       <c r="C38" s="14" t="n">
-        <v>3.5</v>
+        <v>76.5</v>
       </c>
       <c r="D38" s="12" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E38" s="15">
         <f>C38*D38</f>
@@ -1065,19 +1060,19 @@
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>Gaveta Interna c/ Contra Frente</t>
+          <t>Dobradiça Aço s/ Amort. Reta / Baixa</t>
         </is>
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>2.0095C.734.Branco</t>
+          <t>1.1086.000</t>
         </is>
       </c>
       <c r="C39" s="14" t="n">
-        <v>0</v>
+        <v>3.5</v>
       </c>
       <c r="D39" s="12" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E39" s="15">
         <f>C39*D39</f>
@@ -1131,12 +1126,12 @@
     <row r="42">
       <c r="A42" s="12" t="inlineStr">
         <is>
-          <t>Sapateira com contra-frente</t>
+          <t>Gaveta Interna c/ Contra Frente</t>
         </is>
       </c>
       <c r="B42" s="12" t="inlineStr">
         <is>
-          <t>2.0295.720.Branco</t>
+          <t>2.0095C.734.Branco</t>
         </is>
       </c>
       <c r="C42" s="14" t="n">
@@ -1175,12 +1170,12 @@
     <row r="44">
       <c r="A44" s="12" t="inlineStr">
         <is>
-          <t>Gaveta Interna c/ Contra Frente</t>
+          <t>Sapateira com contra-frente</t>
         </is>
       </c>
       <c r="B44" s="12" t="inlineStr">
         <is>
-          <t>2.0095C.734.Branco</t>
+          <t>2.0295.720.Branco</t>
         </is>
       </c>
       <c r="C44" s="14" t="n">
@@ -1241,12 +1236,12 @@
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t>Sapateira com contra-frente</t>
+          <t>Gaveta Interna c/ Contra Frente</t>
         </is>
       </c>
       <c r="B47" s="12" t="inlineStr">
         <is>
-          <t>2.0295.720.Branco</t>
+          <t>2.0095C.734.Branco</t>
         </is>
       </c>
       <c r="C47" s="14" t="n">
@@ -1285,12 +1280,12 @@
     <row r="49">
       <c r="A49" s="12" t="inlineStr">
         <is>
-          <t>Fechamento p/ Armário</t>
+          <t>Sapateira com contra-frente</t>
         </is>
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>2.0135.30.Duratex.Essencial.Rosa Infinito</t>
+          <t>2.0295.720.Branco</t>
         </is>
       </c>
       <c r="C49" s="14" t="n">
@@ -1307,71 +1302,93 @@
     <row r="50">
       <c r="A50" s="12" t="inlineStr">
         <is>
-          <t>Processo de Fabricação</t>
+          <t>Fechamento p/ Armário</t>
         </is>
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>Porta Provençal Configurável</t>
+          <t>2.0135.30.Duratex.Essencial.Rosa Infinito</t>
         </is>
       </c>
       <c r="C50" s="14" t="n">
-        <v>365.51</v>
+        <v>0</v>
       </c>
       <c r="D50" s="12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E50" s="15">
         <f>C50*D50</f>
         <v/>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="16" t="inlineStr">
-        <is>
-          <t>Custo Material Total</t>
-        </is>
-      </c>
-      <c r="B52" s="17">
-        <f>SUM(F18:F21)+SUM(D25:D28)+SUM(E32:E50)</f>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>Processo de Fabricação</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>Porta Provençal Configurável</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="n">
+        <v>365.51</v>
+      </c>
+      <c r="D51" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E51" s="15">
+        <f>C51*D51</f>
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="16" t="inlineStr">
         <is>
-          <t>Preco Venda Material (x Markup)</t>
+          <t>Custo Material Total</t>
         </is>
       </c>
       <c r="B53" s="17">
-        <f>B52*$B$10</f>
+        <f>SUM(F19:F22)+SUM(D26:D29)+SUM(E33:E51)</f>
         <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="16" t="inlineStr">
         <is>
+          <t>Preco Venda Material (x Markup)</t>
+        </is>
+      </c>
+      <c r="B54" s="17">
+        <f>B53*$B$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
           <t>Mao de Obra (Custo Hora x Horas)</t>
         </is>
       </c>
-      <c r="B54" s="17">
-        <f>$B$13*$B$14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="18" t="inlineStr">
+      <c r="B55" s="17">
+        <f>$B$14*$B$15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="18" t="inlineStr">
         <is>
           <t>TOTAL GERAL</t>
         </is>
       </c>
-      <c r="B55" s="19">
-        <f>B53+B54</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="20" t="inlineStr">
+      <c r="B56" s="19">
+        <f>B54+B55</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="20" t="inlineStr">
         <is>
           <t>Legenda: celulas em AZUL sao editaveis (precos, %, horas). O resto recalcula sozinho.</t>
         </is>

</xml_diff>